<commit_message>
Target Q4 pilar Pengadaan Corporate, Maintenance Corporate, Sewa, ISP
Dashboard dasar diganti file user (target 4 pilar di Scoreboard); target ikut
ke app (data/target) sehingga % pencapaian 4 pilar tampil di tab Scoreboard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011hujK4HgUXgzPFn4xuignB
</commit_message>
<xml_diff>
--- a/data/target/target_mflash_Q4_2026.xlsx
+++ b/data/target/target_mflash_Q4_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Cabang</t>
   </si>
@@ -30,6 +30,18 @@
   </si>
   <si>
     <t>Target Corporate</t>
+  </si>
+  <si>
+    <t>Target Pengadaan Corporate</t>
+  </si>
+  <si>
+    <t>Target Maintenance Corporate</t>
+  </si>
+  <si>
+    <t>Target Sewa</t>
+  </si>
+  <si>
+    <t>Target ISP</t>
   </si>
   <si>
     <t>KLENDER</t>
@@ -427,10 +439,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,10 +458,22 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>931426649</v>
@@ -463,10 +487,22 @@
       <c r="E2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>385591373.9104627</v>
+      </c>
+      <c r="G2">
+        <v>12541714.86797358</v>
+      </c>
+      <c r="H2">
+        <v>36953267.02170786</v>
+      </c>
+      <c r="I2">
+        <v>3583347.105135308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>908708926</v>
@@ -480,10 +516,22 @@
       <c r="E3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>436376579.2547675</v>
+      </c>
+      <c r="G3">
+        <v>12235819.38338886</v>
+      </c>
+      <c r="H3">
+        <v>36051967.82605645</v>
+      </c>
+      <c r="I3">
+        <v>3495948.395253959</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>965503234</v>
@@ -497,10 +545,22 @@
       <c r="E4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>399698375.3949919</v>
+      </c>
+      <c r="G4">
+        <v>13000558.09485066</v>
+      </c>
+      <c r="H4">
+        <v>38305215.81518498</v>
+      </c>
+      <c r="I4">
+        <v>3714445.169957331</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>376677804</v>
@@ -514,10 +574,22 @@
       <c r="E5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5">
+        <v>338568035.628699</v>
+      </c>
+      <c r="G5">
+        <v>6882648.403156231</v>
+      </c>
+      <c r="H5">
+        <v>20279231.90215675</v>
+      </c>
+      <c r="I5">
+        <v>1966470.972330352</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>806479172</v>
@@ -531,10 +603,22 @@
       <c r="E6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6">
+        <v>400638842.1606271</v>
+      </c>
+      <c r="G6">
+        <v>10859289.70275761</v>
+      </c>
+      <c r="H6">
+        <v>31996121.4456251</v>
+      </c>
+      <c r="I6">
+        <v>3102654.200787888</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <v>583649036</v>
@@ -548,10 +632,22 @@
       <c r="E7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>387942540.8245509</v>
+      </c>
+      <c r="G7">
+        <v>8412125.826079838</v>
+      </c>
+      <c r="H7">
+        <v>24785727.88041381</v>
+      </c>
+      <c r="I7">
+        <v>2403464.521737097</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>795120310</v>
@@ -565,10 +661,22 @@
       <c r="E8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>481441679.6686803</v>
+      </c>
+      <c r="G8">
+        <v>10706341.96046525</v>
+      </c>
+      <c r="H8">
+        <v>31545471.84779939</v>
+      </c>
+      <c r="I8">
+        <v>3058954.845847214</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>616928602</v>
@@ -582,10 +690,22 @@
       <c r="E9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>702998907.312368</v>
+      </c>
+      <c r="G9">
+        <v>9941603.249003446</v>
+      </c>
+      <c r="H9">
+        <v>29292223.85867087</v>
+      </c>
+      <c r="I9">
+        <v>2840458.071143841</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <v>795120310</v>
@@ -599,10 +719,22 @@
       <c r="E10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>394996041.5668155</v>
+      </c>
+      <c r="G10">
+        <v>10706341.96046525</v>
+      </c>
+      <c r="H10">
+        <v>31545471.84779939</v>
+      </c>
+      <c r="I10">
+        <v>3058954.845847214</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>591884384</v>
@@ -616,10 +748,22 @@
       <c r="E11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>451424047.504932</v>
+      </c>
+      <c r="G11">
+        <v>9176864.537541643</v>
+      </c>
+      <c r="H11">
+        <v>27038975.86954233</v>
+      </c>
+      <c r="I11">
+        <v>2621961.296440469</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <v>468754602</v>
@@ -633,10 +777,22 @@
       <c r="E12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12">
+        <v>526661388.755754</v>
+      </c>
+      <c r="G12">
+        <v>8565073.568372199</v>
+      </c>
+      <c r="H12">
+        <v>25236377.47823951</v>
+      </c>
+      <c r="I12">
+        <v>2447163.876677771</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <v>533866494</v>
@@ -650,10 +806,22 @@
       <c r="E13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13">
+        <v>397817441.8637213</v>
+      </c>
+      <c r="G13">
+        <v>7188543.887740953</v>
+      </c>
+      <c r="H13">
+        <v>21180531.09780816</v>
+      </c>
+      <c r="I13">
+        <v>2053869.682211701</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B14">
         <v>745473038</v>
@@ -667,10 +835,22 @@
       <c r="E14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14">
+        <v>381829506.8479217</v>
+      </c>
+      <c r="G14">
+        <v>8870969.05295692</v>
+      </c>
+      <c r="H14">
+        <v>26137676.67389093</v>
+      </c>
+      <c r="I14">
+        <v>2534562.58655912</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B15">
         <v>454364463</v>
@@ -684,10 +864,22 @@
       <c r="E15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15">
+        <v>413805376.879521</v>
+      </c>
+      <c r="G15">
+        <v>6117909.691694428</v>
+      </c>
+      <c r="H15">
+        <v>18025983.91302823</v>
+      </c>
+      <c r="I15">
+        <v>1747974.197626979</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B16">
         <v>545225356</v>
@@ -701,10 +893,22 @@
       <c r="E16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16">
+        <v>451424047.504932</v>
+      </c>
+      <c r="G16">
+        <v>7341491.630033313</v>
+      </c>
+      <c r="H16">
+        <v>21631180.69563387</v>
+      </c>
+      <c r="I16">
+        <v>2097569.037152375</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <v>686369913</v>
@@ -718,10 +922,22 @@
       <c r="E17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17">
+        <v>362079704.7695809</v>
+      </c>
+      <c r="G17">
+        <v>8412125.826079838</v>
+      </c>
+      <c r="H17">
+        <v>24785727.88041381</v>
+      </c>
+      <c r="I17">
+        <v>2403464.521737097</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <v>397560155</v>
@@ -735,10 +951,22 @@
       <c r="E18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18">
+        <v>691243072.7419271</v>
+      </c>
+      <c r="G18">
+        <v>5353170.980232624</v>
+      </c>
+      <c r="H18">
+        <v>15772735.9238997</v>
+      </c>
+      <c r="I18">
+        <v>1529477.422923607</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B19">
         <v>391880724</v>
@@ -752,10 +980,22 @@
       <c r="E19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19">
+        <v>681368171.7027568</v>
+      </c>
+      <c r="G19">
+        <v>5276697.109086444</v>
+      </c>
+      <c r="H19">
+        <v>15547411.12498684</v>
+      </c>
+      <c r="I19">
+        <v>1507627.74545327</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <v>261253816</v>
@@ -768,6 +1008,18 @@
       </c>
       <c r="E20">
         <v>0</v>
+      </c>
+      <c r="F20">
+        <v>365559431.8024313</v>
+      </c>
+      <c r="G20">
+        <v>3517798.072724296</v>
+      </c>
+      <c r="H20">
+        <v>10364940.74999123</v>
+      </c>
+      <c r="I20">
+        <v>1005085.163635513</v>
       </c>
     </row>
   </sheetData>
@@ -782,17 +1034,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>